<commit_message>
Updates to explainer file
</commit_message>
<xml_diff>
--- a/Presentations/LAMBDA function Explainer.xlsx
+++ b/Presentations/LAMBDA function Explainer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\local_python\Statistical_Analysis_Lambda_Catalog\Presentations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LocalPython\Statistical_Analysis_Lambda_Catalog\Presentations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E428EFAB-6FFD-4216-AF88-15FA4A449B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFA0F3C-AC97-46CD-B9A3-328F410AE7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{472FB111-C493-4DBD-9493-F95C4CD26A08}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{472FB111-C493-4DBD-9493-F95C4CD26A08}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Side 1</t>
   </si>
@@ -92,12 +92,15 @@
   <si>
     <t>LAMBDA Hypotenuse</t>
   </si>
+  <si>
+    <t>Let example</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,14 +129,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -212,15 +217,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{77F366B0-8EBB-4C08-B654-38EBDDF16307}" name="Right_Triangles" displayName="Right_Triangles" ref="A1:D4" totalsRowShown="0">
-  <autoFilter ref="A1:D4" xr:uid="{77F366B0-8EBB-4C08-B654-38EBDDF16307}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{77F366B0-8EBB-4C08-B654-38EBDDF16307}" name="Right_Triangles" displayName="Right_Triangles" ref="A1:E4" totalsRowShown="0">
+  <autoFilter ref="A1:E4" xr:uid="{77F366B0-8EBB-4C08-B654-38EBDDF16307}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{5F5D5EA7-E327-47EB-850E-83A1FBD22A00}" name="Side 1"/>
     <tableColumn id="2" xr3:uid="{4A0C7AC5-3595-4AFC-A558-EE84B337D4A0}" name="Side 2"/>
-    <tableColumn id="3" xr3:uid="{639BB46B-CC4A-4EA8-B0D9-EFAF54C88360}" name="Hypotenuse" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{639BB46B-CC4A-4EA8-B0D9-EFAF54C88360}" name="Hypotenuse" dataDxfId="2">
       <calculatedColumnFormula>SQRT(Right_Triangles[[#This Row],[Side 1]]^2+Right_Triangles[[#This Row],[Side 2]]^2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{364E7ECA-FE13-43C7-B31D-536D36EBAF9F}" name="LAMBDA Hypotenuse" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{ABA06F8F-BC40-4F75-AA0C-F22837FEF89D}" name="Let example" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.LET(_xlpm.a_square, Right_Triangles[[#This Row],[Side 1]]^2, _xlpm.b_squared, Right_Triangles[[#This Row],[Side 2]]^2, SQRT(_xlpm.a_square+_xlpm.b_squared))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{364E7ECA-FE13-43C7-B31D-536D36EBAF9F}" name="LAMBDA Hypotenuse" dataDxfId="1">
       <calculatedColumnFormula array="1">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -545,14 +553,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E0F324A-7B8F-4297-9FA9-044B0111068A}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.375" customWidth="1"/>
-    <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="22" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -563,10 +573,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>3</v>
       </c>
@@ -577,16 +590,20 @@
         <f>SQRT(Right_Triangles[[#This Row],[Side 1]]^2+Right_Triangles[[#This Row],[Side 2]]^2)</f>
         <v>5</v>
       </c>
-      <c r="D2" cm="1">
-        <f t="array" ref="D2">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
+      <c r="D2">
+        <f>_xlfn.LET(_xlpm.a_square, Right_Triangles[[#This Row],[Side 1]]^2, _xlpm.b_squared, Right_Triangles[[#This Row],[Side 2]]^2, SQRT(_xlpm.a_square+_xlpm.b_squared))</f>
         <v>5</v>
       </c>
-      <c r="F2" cm="1">
-        <f t="array" ref="F2">_xlfn.LAMBDA(_xlpm.a,_xlpm.b, SQRT(_xlpm.a^2+_xlpm.b^2))(3,4)</f>
+      <c r="E2" cm="1">
+        <f t="array" ref="E2">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
         <v>5</v>
       </c>
+      <c r="G2" cm="1">
+        <f t="array" ref="G2">_xlfn.LAMBDA(_xlpm.a,_xlpm.b, SQRT(_xlpm.a^2+_xlpm.b^2))(3,4)</f>
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>5</v>
       </c>
@@ -597,33 +614,47 @@
         <f>SQRT(Right_Triangles[[#This Row],[Side 1]]^2+Right_Triangles[[#This Row],[Side 2]]^2)</f>
         <v>13</v>
       </c>
-      <c r="D3" cm="1">
-        <f t="array" ref="D3">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
+      <c r="D3">
+        <f>_xlfn.LET(_xlpm.a_square, Right_Triangles[[#This Row],[Side 1]]^2, _xlpm.b_squared, Right_Triangles[[#This Row],[Side 2]]^2, SQRT(_xlpm.a_square+_xlpm.b_squared))</f>
         <v>13</v>
       </c>
-      <c r="F3" t="e" cm="1" vm="1">
-        <f t="array" ref="F3">_xlfn.LAMBDA(_xlpm.a,_xlpm.b, SQRT(_xlpm.a^2+_xlpm.b^2))</f>
+      <c r="E3" cm="1">
+        <f t="array" ref="E3">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
+        <v>13</v>
+      </c>
+      <c r="G3" t="e" cm="1" vm="1">
+        <f t="array" ref="G3">_xlfn.LAMBDA(_xlpm.a,_xlpm.b, SQRT(_xlpm.a^2+_xlpm.b^2))</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>20</v>
       </c>
       <c r="B4">
         <v>21</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <f>SQRT(Right_Triangles[[#This Row],[Side 1]]^2+Right_Triangles[[#This Row],[Side 2]]^2)</f>
         <v>29</v>
       </c>
-      <c r="D4" cm="1">
-        <f t="array" ref="D4">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
+      <c r="D4">
+        <f>_xlfn.LET(_xlpm.a_square, Right_Triangles[[#This Row],[Side 1]]^2, _xlpm.b_squared, Right_Triangles[[#This Row],[Side 2]]^2, SQRT(_xlpm.a_square+_xlpm.b_squared))</f>
         <v>29</v>
       </c>
-      <c r="F4" cm="1">
-        <f t="array" ref="F4">Hypotenuse(3,4)</f>
+      <c r="E4" cm="1">
+        <f t="array" ref="E4">Hypotenuse(Right_Triangles[[#This Row],[Side 1]],Right_Triangles[[#This Row],[Side 2]])</f>
+        <v>29</v>
+      </c>
+      <c r="G4" cm="1">
+        <f t="array" ref="G4">Hypotenuse(3,4)</f>
         <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G5">
+        <f>SUMSQ(A2,B2)</f>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>